<commit_message>
feat: update expert fields and Russian templates
- Increase expert position field from 300 to 500 chars
- Add dd_comments field for communication notes
- Make expertise_tags optional for experts
- Add Russian field name mappings in expert upload
- Update all templates to use Russian headers (Имя, Телеграм, etc.)
- Update test data generation script with new expert fields
- Regenerate test data files with Russian headers
</commit_message>
<xml_diff>
--- a/data/import_ready/experts.xlsx
+++ b/data/import_ready/experts.xlsx
@@ -413,28 +413,38 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>name *</t>
+          <t>Имя *</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>telegram</t>
+          <t>Телеграм</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>position</t>
+          <t>Описание</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>expertise_tags</t>
+          <t>Тематики</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Статус</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Комментарии</t>
         </is>
       </c>
     </row>
@@ -451,12 +461,22 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Senior ML Engineer</t>
+          <t>Senior ML Engineer в TechCorp, 8 лет опыта</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>NLP, CV, ML</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Подтвердил</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Готов взять NLP и CV проекты</t>
         </is>
       </c>
     </row>
@@ -473,7 +493,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Head of AI Research</t>
+          <t>Head of AI Research в UniversityLab</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -481,6 +501,12 @@
           <t>NLP, Research, Education</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Подтвердил</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -495,12 +521,22 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Computer Vision Lead</t>
+          <t>Computer Vision Lead, специализация медицина</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
           <t>CV, Deep Learning</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Подтвердил</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Интересуют прикладные CV проекты</t>
         </is>
       </c>
     </row>
@@ -517,12 +553,22 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>FinTech Product Manager</t>
+          <t>FinTech Product Manager в банке</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
           <t>Finance, Product</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Уточняется</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Написала, что постарается приехать</t>
         </is>
       </c>
     </row>
@@ -539,7 +585,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>EdTech Founder</t>
+          <t>EdTech Founder, бывший преподаватель ВШЭ</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -547,6 +593,12 @@
           <t>Education, Startups</t>
         </is>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Подтвердил</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -561,12 +613,22 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ML Team Lead</t>
+          <t>ML Team Lead в e-commerce</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
           <t>ML, Data Science</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Подтвердил</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Recsys, fintech могу взять</t>
         </is>
       </c>
     </row>
@@ -583,7 +645,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Senior Frontend Dev</t>
+          <t>Senior Frontend Dev, React/Vue эксперт</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -591,6 +653,12 @@
           <t>Web, UI/UX</t>
         </is>
       </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Не ответил</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -605,7 +673,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Mobile Dev Lead</t>
+          <t>Mobile Dev Lead в стартапе</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -613,6 +681,12 @@
           <t>Mobile, iOS, Android</t>
         </is>
       </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Подтвердил</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -627,12 +701,22 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Backend Architect</t>
+          <t>Backend Architect, highload системы</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
           <t>Backend, Databases, API</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Подтвердил</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Могу помочь с архитектурой</t>
         </is>
       </c>
     </row>
@@ -649,12 +733,22 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Data Scientist в консалтинге</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
           <t>Data Science, Analytics, ML</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Отказался</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Занята в этот день</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: replace Тематики with Теги and Имя with ФИО for consistency
</commit_message>
<xml_diff>
--- a/data/import_ready/experts.xlsx
+++ b/data/import_ready/experts.xlsx
@@ -419,7 +419,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Имя *</t>
+          <t>ФИО *</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -434,7 +434,7 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Тематики</t>
+          <t>Теги</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">

</xml_diff>